<commit_message>
Intégration réseau v12 : CTA 5 décalée pour la porte de la terrasse
- files/b3d : gaines.json et equip.json v12 (GAI_V=3, EQ_V=8)
- files/gaines : reseaux.png et Excel, docs/*.b64.txt à jour
- Réservations : 83 (55 murs, 14 trémies, 14 poutres)
- Implantation : image et explication du décalage sur la fiche CTA 5
- SYN-03 B : CTA 5 à -68,93 / 39,2, 69 Pa, réseau v12
- CONTEXTE.md : journal

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013DW4zPTHhjq33S132qLfm8
</commit_message>
<xml_diff>
--- a/files/gaines/EHPAD_Dimensionnement_Gaines.xlsx
+++ b/files/gaines/EHPAD_Dimensionnement_Gaines.xlsx
@@ -1258,10 +1258,10 @@
     <t xml:space="preserve">CTA5-R48</t>
   </si>
   <si>
+    <t xml:space="preserve">CTA5-R49</t>
+  </si>
+  <si>
     <t xml:space="preserve">LOG10 vêtements, BUR01 bur. mut., SOI03 soins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CTA5-R49</t>
   </si>
   <si>
     <t xml:space="preserve">CTA5-R50</t>
@@ -2229,11 +2229,11 @@
       </c>
       <c r="I9" s="10" t="n">
         <f aca="false">SUMIF(Tronçons!$A$5:$A$280,A9,Tronçons!$G$5:$G$280)</f>
-        <v>194.1</v>
+        <v>190.1</v>
       </c>
       <c r="J9" s="10" t="n">
         <f aca="false">MAX(SUMIFS(Tronçons!$T$5:$T$280,Tronçons!$A$5:$A$280,A9,Tronçons!$U$5:$U$280,"X",Tronçons!$E$5:$E$280,"Soufflage"),SUMIFS(Tronçons!$T$5:$T$280,Tronçons!$A$5:$A$280,A9,Tronçons!$U$5:$U$280,"X",Tronçons!$E$5:$E$280,"Reprise"))</f>
-        <v>70.6540353156577</v>
+        <v>68.6229176337802</v>
       </c>
       <c r="K9" s="5" t="n">
         <f aca="false">COUNTIFS(Tronçons!$A$5:$A$280,A9,Tronçons!$O$5:$O$280,"NON")</f>
@@ -18421,7 +18421,7 @@
         <v>100</v>
       </c>
       <c r="G199" s="22" t="n">
-        <v>5.35</v>
+        <v>3.95</v>
       </c>
       <c r="H199" s="6" t="n">
         <v>6123</v>
@@ -18472,7 +18472,7 @@
       </c>
       <c r="T199" s="23" t="n">
         <f aca="false">S199*G199*(1+Hypothèses!$B$22)</f>
-        <v>4.67812474542168</v>
+        <v>3.45394256904965</v>
       </c>
       <c r="U199" s="5" t="s">
         <v>101</v>
@@ -18659,7 +18659,7 @@
       </c>
       <c r="F202" s="21"/>
       <c r="G202" s="22" t="n">
-        <v>1.9</v>
+        <v>1.3</v>
       </c>
       <c r="H202" s="6" t="n">
         <v>6123</v>
@@ -18710,7 +18710,7 @@
       </c>
       <c r="T202" s="23" t="n">
         <f aca="false">S202*G202*(1+Hypothèses!$B$22)</f>
-        <v>1.66139009650489</v>
+        <v>1.13674059234545</v>
       </c>
       <c r="U202" s="5" t="s">
         <v>101</v>
@@ -21940,7 +21940,7 @@
         <v>100</v>
       </c>
       <c r="G243" s="22" t="n">
-        <v>4.35</v>
+        <v>3</v>
       </c>
       <c r="H243" s="6" t="n">
         <v>6123</v>
@@ -21991,7 +21991,7 @@
       </c>
       <c r="T243" s="23" t="n">
         <f aca="false">S243*G243*(1+Hypothèses!$B$22)</f>
-        <v>3.80370890515594</v>
+        <v>2.6232475207972</v>
       </c>
       <c r="U243" s="5" t="s">
         <v>101</v>
@@ -22176,11 +22176,9 @@
       <c r="E246" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="F246" s="21" t="s">
-        <v>387</v>
-      </c>
+      <c r="F246" s="21"/>
       <c r="G246" s="22" t="n">
-        <v>1.3</v>
+        <v>2.2</v>
       </c>
       <c r="H246" s="6" t="n">
         <v>6123</v>
@@ -22231,7 +22229,7 @@
       </c>
       <c r="T246" s="23" t="n">
         <f aca="false">S246*G246*(1+Hypothèses!$B$22)</f>
-        <v>1.13674059234545</v>
+        <v>1.92371484858461</v>
       </c>
       <c r="U246" s="5" t="s">
         <v>101</v>
@@ -22246,7 +22244,7 @@
         <v>27</v>
       </c>
       <c r="B247" s="21" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C247" s="21" t="s">
         <v>108</v>
@@ -22257,12 +22255,14 @@
       <c r="E247" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="F247" s="21"/>
+      <c r="F247" s="21" t="s">
+        <v>388</v>
+      </c>
       <c r="G247" s="22" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="H247" s="6" t="n">
-        <v>5994</v>
+        <v>6123</v>
       </c>
       <c r="I247" s="23" t="n">
         <f aca="false">IF(A247="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H247,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H247,Hypothèses!$A$6:$A$16,1)))</f>
@@ -22270,7 +22270,7 @@
       </c>
       <c r="J247" s="24" t="n">
         <f aca="false">H247/3600/I247</f>
-        <v>0.2775</v>
+        <v>0.283472222222222</v>
       </c>
       <c r="K247" s="21" t="n">
         <f aca="false">IF(A247="CTA 4",Hypothèses!$B$25,IF(AND(A247="CTA 5",H247&gt;4000),Hypothèses!$B$29,IF(H247&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -22278,15 +22278,15 @@
       </c>
       <c r="L247" s="21" t="n">
         <f aca="false">MAX(Hypothèses!$B$26,CEILING(J247/(K247/1000)*1000,Hypothèses!$B$27))</f>
-        <v>800</v>
+        <v>850</v>
       </c>
       <c r="M247" s="24" t="n">
         <f aca="false">L247*K247/1000000</f>
-        <v>0.28</v>
+        <v>0.2975</v>
       </c>
       <c r="N247" s="25" t="n">
         <f aca="false">H247/3600/M247</f>
-        <v>5.94642857142857</v>
+        <v>5.71708683473389</v>
       </c>
       <c r="O247" s="21" t="str">
         <f aca="false">IF(N247&lt;=I247,"oui","NON")</f>
@@ -22294,23 +22294,23 @@
       </c>
       <c r="P247" s="24" t="n">
         <f aca="false">1.3*((L247/1000)*(K247/1000))^0.625/((L247/1000)+(K247/1000))^0.25</f>
-        <v>0.566555763342023</v>
+        <v>0.582206965594154</v>
       </c>
       <c r="Q247" s="26" t="n">
         <f aca="false">N247*P247/Hypothèses!$B$20</f>
-        <v>224598.891896302</v>
+        <v>221901.851872581</v>
       </c>
       <c r="R247" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P247)+5.74/Q247^0.9))^2</f>
-        <v>0.0173303541791289</v>
+        <v>0.0173062640953008</v>
       </c>
       <c r="S247" s="25" t="n">
         <f aca="false">R247/P247*Hypothèses!$B$19*N247^2/2</f>
-        <v>0.648975706690844</v>
+        <v>0.582943893510489</v>
       </c>
       <c r="T247" s="23" t="n">
         <f aca="false">S247*G247*(1+Hypothèses!$B$22)</f>
-        <v>1.4601953400544</v>
+        <v>1.13674059234545</v>
       </c>
       <c r="U247" s="5" t="s">
         <v>101</v>
@@ -22340,7 +22340,7 @@
         <v>390</v>
       </c>
       <c r="G248" s="22" t="n">
-        <v>2.225</v>
+        <v>0.875</v>
       </c>
       <c r="H248" s="6" t="n">
         <v>5994</v>
@@ -22391,7 +22391,7 @@
       </c>
       <c r="T248" s="23" t="n">
         <f aca="false">S248*G248*(1+Hypothèses!$B$22)</f>
-        <v>2.16595642108069</v>
+        <v>0.851780615031733</v>
       </c>
       <c r="U248" s="5" t="s">
         <v>101</v>

</xml_diff>

<commit_message>
Intégration réseau v13 : onglet Bouches, antennes dans la 3D, quantités de bouches au devis
- gaines.json (1 540 objets avec antennes) et equip.json recopiés (GAI_V 4, EQ_V 9)
- bouches.json, Excel et plan des bouches dans files/bouches/, documents ajoutés aux tâches i05 et i02
- Onglet Bouches : débits par CTA, plan, tableau filtrable, vitesse au col, export CSV
- 3D : antennes plus claires et masquables, fiche avec la bouche desservie
- Devis : une ligne par type de bouche

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HnQUSWdbuW1WHe65pTp6tB
</commit_message>
<xml_diff>
--- a/files/gaines/EHPAD_Dimensionnement_Gaines.xlsx
+++ b/files/gaines/EHPAD_Dimensionnement_Gaines.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Tronçons" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tronçons!$A$4:$V$280</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tronçons!$A$4:$V$279</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -95,7 +95,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1952" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1943" uniqueCount="427">
   <si>
     <t xml:space="preserve">Gaines principales de ventilation – synthèse par CTA</t>
   </si>
@@ -301,7 +301,7 @@
     <t xml:space="preserve">• Tracé v2 : chaque CTA est posée juste au-dessus de sa descente. CTA 1, 2 et 5 : gaine technique créée dans un local annexe (ménage, office) car le DCE n'a que des gaines de désenfumage. CTA 3 et 4 (étage seul) : descente directe par la toiture dans le couloir.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Gaines horizontales uniquement dans les couloirs (et le hall / la salle à manger pour la CTA 5), parallèles aux murs, changements de direction à 90°. Axe des gaines à 2,78 m (RDC) et 6,14 m (étage) ; CTA 5 : 2,765 m (RDC) et 6,09 m (étage).</t>
+    <t xml:space="preserve">• Gaines horizontales uniquement dans les couloirs (et le hall / la salle à manger pour la CTA 5), parallèles aux murs, changements de direction à 90°. Axe des gaines à 2,78 m (RDC) et 6,14 m (étage) ; CTA 5 : 2,765 m (RDC) et 6,09 m (étage). CTA 3 et 4 : soufflage et reprise écartés de 1,0 m et 0,7 m pour laisser passer les antennes des bouches. CTA 5 RDC : la reprise passe au-dessus du faux plafond des bureaux côté sud (y = 34,4 m), le couloir garde seulement le soufflage.</t>
   </si>
   <si>
     <t xml:space="preserve">• Débits : 90 m³/h soufflés par chambre et 90 m³/h repris par salle de bains (CCTP § 2.2 et § 4.10) ; locaux communs : onglet « Débits par local » du fichier des débits.</t>
@@ -1258,12 +1258,12 @@
     <t xml:space="preserve">CTA5-R48</t>
   </si>
   <si>
+    <t xml:space="preserve">LOG10 vêtements, BUR01 bur. mut., LOG02 chariots, SOI03 soins</t>
+  </si>
+  <si>
     <t xml:space="preserve">CTA5-R49</t>
   </si>
   <si>
-    <t xml:space="preserve">LOG10 vêtements, BUR01 bur. mut., SOI03 soins</t>
-  </si>
-  <si>
     <t xml:space="preserve">CTA5-R50</t>
   </si>
   <si>
@@ -1294,6 +1294,9 @@
     <t xml:space="preserve">CTA5-R58</t>
   </si>
   <si>
+    <t xml:space="preserve">BUR01 bur. cadre, SOI02 prépa., SOI05 transmissions</t>
+  </si>
+  <si>
     <t xml:space="preserve">CTA5-R59</t>
   </si>
   <si>
@@ -1312,21 +1315,21 @@
     <t xml:space="preserve">CTA5-R64</t>
   </si>
   <si>
+    <t xml:space="preserve">LOG02 chariots, BUR02 accueil</t>
+  </si>
+  <si>
     <t xml:space="preserve">CTA5-R65</t>
   </si>
   <si>
-    <t xml:space="preserve">LOG02 chariots, BUR02 accueil</t>
-  </si>
-  <si>
     <t xml:space="preserve">CTA5-R66</t>
   </si>
   <si>
+    <t xml:space="preserve">LOG06 linge P, LOG03 réserve magasin, BUR02A b. animation, VIE06 coiffure, LOG02 stock</t>
+  </si>
+  <si>
     <t xml:space="preserve">CTA5-R67</t>
   </si>
   <si>
-    <t xml:space="preserve">LOG06 linge P, LOG03 réserve magasin, BUR02A b. animation, VIE06 coiffure, LOG02 stock</t>
-  </si>
-  <si>
     <t xml:space="preserve">CTA5-R68</t>
   </si>
   <si>
@@ -1360,19 +1363,16 @@
     <t xml:space="preserve">CTA5-R78</t>
   </si>
   <si>
+    <t xml:space="preserve">BUR06 bureau, LOG03 réserve magasin, LOG03 réserve magasin, LOG03 réserve matériel, HEB03 salle à manger salon, LOG02 ch</t>
+  </si>
+  <si>
     <t xml:space="preserve">CTA5-R79</t>
   </si>
   <si>
-    <t xml:space="preserve">BUR06 bureau, LOG03 réserve magasin, LOG03 réserve magasin, LOG03 réserve matériel, HEB03 salle à manger salon, LOG02 ch</t>
-  </si>
-  <si>
     <t xml:space="preserve">CTA5-R80</t>
   </si>
   <si>
     <t xml:space="preserve">CTA5-R81</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CTA5-R82</t>
   </si>
   <si>
     <t xml:space="preserve">HEB03 salle à manger salon, DET01 détente</t>
@@ -2024,23 +2024,23 @@
         <v>5.18518518518518</v>
       </c>
       <c r="H5" s="5" t="n">
-        <f aca="false">COUNTIF(Tronçons!$A$5:$A$280,A5)</f>
+        <f aca="false">COUNTIF(Tronçons!$A$5:$A$279,A5)</f>
         <v>70</v>
       </c>
       <c r="I5" s="10" t="n">
-        <f aca="false">SUMIF(Tronçons!$A$5:$A$280,A5,Tronçons!$G$5:$G$280)</f>
+        <f aca="false">SUMIF(Tronçons!$A$5:$A$279,A5,Tronçons!$G$5:$G$279)</f>
         <v>150.78</v>
       </c>
       <c r="J5" s="10" t="n">
-        <f aca="false">MAX(SUMIFS(Tronçons!$T$5:$T$280,Tronçons!$A$5:$A$280,A5,Tronçons!$U$5:$U$280,"X",Tronçons!$E$5:$E$280,"Soufflage"),SUMIFS(Tronçons!$T$5:$T$280,Tronçons!$A$5:$A$280,A5,Tronçons!$U$5:$U$280,"X",Tronçons!$E$5:$E$280,"Reprise"))</f>
+        <f aca="false">MAX(SUMIFS(Tronçons!$T$5:$T$279,Tronçons!$A$5:$A$279,A5,Tronçons!$U$5:$U$279,"X",Tronçons!$E$5:$E$279,"Soufflage"),SUMIFS(Tronçons!$T$5:$T$279,Tronçons!$A$5:$A$279,A5,Tronçons!$U$5:$U$279,"X",Tronçons!$E$5:$E$279,"Reprise"))</f>
         <v>36.3258207989034</v>
       </c>
       <c r="K5" s="5" t="n">
-        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$280,A5,Tronçons!$O$5:$O$280,"NON")</f>
+        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$279,A5,Tronçons!$O$5:$O$279,"NON")</f>
         <v>0</v>
       </c>
       <c r="L5" s="5" t="n">
-        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$280,A5,Tronçons!$V$5:$V$280,"NON")</f>
+        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$279,A5,Tronçons!$V$5:$V$279,"NON")</f>
         <v>0</v>
       </c>
       <c r="M5" s="5" t="s">
@@ -2074,23 +2074,23 @@
         <v>5</v>
       </c>
       <c r="H6" s="5" t="n">
-        <f aca="false">COUNTIF(Tronçons!$A$5:$A$280,A6)</f>
+        <f aca="false">COUNTIF(Tronçons!$A$5:$A$279,A6)</f>
         <v>64</v>
       </c>
       <c r="I6" s="10" t="n">
-        <f aca="false">SUMIF(Tronçons!$A$5:$A$280,A6,Tronçons!$G$5:$G$280)</f>
+        <f aca="false">SUMIF(Tronçons!$A$5:$A$279,A6,Tronçons!$G$5:$G$279)</f>
         <v>141.366</v>
       </c>
       <c r="J6" s="10" t="n">
-        <f aca="false">MAX(SUMIFS(Tronçons!$T$5:$T$280,Tronçons!$A$5:$A$280,A6,Tronçons!$U$5:$U$280,"X",Tronçons!$E$5:$E$280,"Soufflage"),SUMIFS(Tronçons!$T$5:$T$280,Tronçons!$A$5:$A$280,A6,Tronçons!$U$5:$U$280,"X",Tronçons!$E$5:$E$280,"Reprise"))</f>
+        <f aca="false">MAX(SUMIFS(Tronçons!$T$5:$T$279,Tronçons!$A$5:$A$279,A6,Tronçons!$U$5:$U$279,"X",Tronçons!$E$5:$E$279,"Soufflage"),SUMIFS(Tronçons!$T$5:$T$279,Tronçons!$A$5:$A$279,A6,Tronçons!$U$5:$U$279,"X",Tronçons!$E$5:$E$279,"Reprise"))</f>
         <v>37.107273515251</v>
       </c>
       <c r="K6" s="5" t="n">
-        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$280,A6,Tronçons!$O$5:$O$280,"NON")</f>
+        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$279,A6,Tronçons!$O$5:$O$279,"NON")</f>
         <v>0</v>
       </c>
       <c r="L6" s="5" t="n">
-        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$280,A6,Tronçons!$V$5:$V$280,"NON")</f>
+        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$279,A6,Tronçons!$V$5:$V$279,"NON")</f>
         <v>0</v>
       </c>
       <c r="M6" s="5" t="s">
@@ -2124,23 +2124,23 @@
         <v>4.33333333333333</v>
       </c>
       <c r="H7" s="5" t="n">
-        <f aca="false">COUNTIF(Tronçons!$A$5:$A$280,A7)</f>
+        <f aca="false">COUNTIF(Tronçons!$A$5:$A$279,A7)</f>
         <v>30</v>
       </c>
       <c r="I7" s="10" t="n">
-        <f aca="false">SUMIF(Tronçons!$A$5:$A$280,A7,Tronçons!$G$5:$G$280)</f>
-        <v>67.14</v>
+        <f aca="false">SUMIF(Tronçons!$A$5:$A$279,A7,Tronçons!$G$5:$G$279)</f>
+        <v>67.19</v>
       </c>
       <c r="J7" s="10" t="n">
-        <f aca="false">MAX(SUMIFS(Tronçons!$T$5:$T$280,Tronçons!$A$5:$A$280,A7,Tronçons!$U$5:$U$280,"X",Tronçons!$E$5:$E$280,"Soufflage"),SUMIFS(Tronçons!$T$5:$T$280,Tronçons!$A$5:$A$280,A7,Tronçons!$U$5:$U$280,"X",Tronçons!$E$5:$E$280,"Reprise"))</f>
-        <v>29.8575047760053</v>
+        <f aca="false">MAX(SUMIFS(Tronçons!$T$5:$T$279,Tronçons!$A$5:$A$279,A7,Tronçons!$U$5:$U$279,"X",Tronçons!$E$5:$E$279,"Soufflage"),SUMIFS(Tronçons!$T$5:$T$279,Tronçons!$A$5:$A$279,A7,Tronçons!$U$5:$U$279,"X",Tronçons!$E$5:$E$279,"Reprise"))</f>
+        <v>30.1869322327972</v>
       </c>
       <c r="K7" s="5" t="n">
-        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$280,A7,Tronçons!$O$5:$O$280,"NON")</f>
+        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$279,A7,Tronçons!$O$5:$O$279,"NON")</f>
         <v>0</v>
       </c>
       <c r="L7" s="5" t="n">
-        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$280,A7,Tronçons!$V$5:$V$280,"NON")</f>
+        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$279,A7,Tronçons!$V$5:$V$279,"NON")</f>
         <v>0</v>
       </c>
       <c r="M7" s="5" t="s">
@@ -2174,23 +2174,23 @@
         <v>4.33333333333333</v>
       </c>
       <c r="H8" s="5" t="n">
-        <f aca="false">COUNTIF(Tronçons!$A$5:$A$280,A8)</f>
+        <f aca="false">COUNTIF(Tronçons!$A$5:$A$279,A8)</f>
         <v>30</v>
       </c>
       <c r="I8" s="10" t="n">
-        <f aca="false">SUMIF(Tronçons!$A$5:$A$280,A8,Tronçons!$G$5:$G$280)</f>
-        <v>66.99</v>
+        <f aca="false">SUMIF(Tronçons!$A$5:$A$279,A8,Tronçons!$G$5:$G$279)</f>
+        <v>67.19</v>
       </c>
       <c r="J8" s="10" t="n">
-        <f aca="false">MAX(SUMIFS(Tronçons!$T$5:$T$280,Tronçons!$A$5:$A$280,A8,Tronçons!$U$5:$U$280,"X",Tronçons!$E$5:$E$280,"Soufflage"),SUMIFS(Tronçons!$T$5:$T$280,Tronçons!$A$5:$A$280,A8,Tronçons!$U$5:$U$280,"X",Tronçons!$E$5:$E$280,"Reprise"))</f>
-        <v>25.1942495709174</v>
+        <f aca="false">MAX(SUMIFS(Tronçons!$T$5:$T$279,Tronçons!$A$5:$A$279,A8,Tronçons!$U$5:$U$279,"X",Tronçons!$E$5:$E$279,"Soufflage"),SUMIFS(Tronçons!$T$5:$T$279,Tronçons!$A$5:$A$279,A8,Tronçons!$U$5:$U$279,"X",Tronçons!$E$5:$E$279,"Reprise"))</f>
+        <v>25.4060243645693</v>
       </c>
       <c r="K8" s="5" t="n">
-        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$280,A8,Tronçons!$O$5:$O$280,"NON")</f>
+        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$279,A8,Tronçons!$O$5:$O$279,"NON")</f>
         <v>0</v>
       </c>
       <c r="L8" s="5" t="n">
-        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$280,A8,Tronçons!$V$5:$V$280,"NON")</f>
+        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$279,A8,Tronçons!$V$5:$V$279,"NON")</f>
         <v>0</v>
       </c>
       <c r="M8" s="5" t="s">
@@ -2224,23 +2224,23 @@
         <v>5.71708683473389</v>
       </c>
       <c r="H9" s="5" t="n">
-        <f aca="false">COUNTIF(Tronçons!$A$5:$A$280,A9)</f>
-        <v>82</v>
+        <f aca="false">COUNTIF(Tronçons!$A$5:$A$279,A9)</f>
+        <v>81</v>
       </c>
       <c r="I9" s="10" t="n">
-        <f aca="false">SUMIF(Tronçons!$A$5:$A$280,A9,Tronçons!$G$5:$G$280)</f>
-        <v>190.1</v>
+        <f aca="false">SUMIF(Tronçons!$A$5:$A$279,A9,Tronçons!$G$5:$G$279)</f>
+        <v>192.9</v>
       </c>
       <c r="J9" s="10" t="n">
-        <f aca="false">MAX(SUMIFS(Tronçons!$T$5:$T$280,Tronçons!$A$5:$A$280,A9,Tronçons!$U$5:$U$280,"X",Tronçons!$E$5:$E$280,"Soufflage"),SUMIFS(Tronçons!$T$5:$T$280,Tronçons!$A$5:$A$280,A9,Tronçons!$U$5:$U$280,"X",Tronçons!$E$5:$E$280,"Reprise"))</f>
-        <v>68.6229176337802</v>
+        <f aca="false">MAX(SUMIFS(Tronçons!$T$5:$T$279,Tronçons!$A$5:$A$279,A9,Tronçons!$U$5:$U$279,"X",Tronçons!$E$5:$E$279,"Soufflage"),SUMIFS(Tronçons!$T$5:$T$279,Tronçons!$A$5:$A$279,A9,Tronçons!$U$5:$U$279,"X",Tronçons!$E$5:$E$279,"Reprise"))</f>
+        <v>71.0422607330011</v>
       </c>
       <c r="K9" s="5" t="n">
-        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$280,A9,Tronçons!$O$5:$O$280,"NON")</f>
+        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$279,A9,Tronçons!$O$5:$O$279,"NON")</f>
         <v>0</v>
       </c>
       <c r="L9" s="5" t="n">
-        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$280,A9,Tronçons!$V$5:$V$280,"NON")</f>
+        <f aca="false">COUNTIFS(Tronçons!$A$5:$A$279,A9,Tronçons!$V$5:$V$279,"NON")</f>
         <v>0</v>
       </c>
       <c r="M9" s="5" t="s">
@@ -2755,7 +2755,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:V280"/>
+  <dimension ref="A1:V279"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -13569,7 +13569,7 @@
         <v>100</v>
       </c>
       <c r="G139" s="22" t="n">
-        <v>2.2</v>
+        <v>1.95</v>
       </c>
       <c r="H139" s="6" t="n">
         <v>1170</v>
@@ -13620,7 +13620,7 @@
       </c>
       <c r="T139" s="23" t="n">
         <f aca="false">S139*G139*(1+Hypothèses!$B$22)</f>
-        <v>2.58835858907914</v>
+        <v>2.29422693122923</v>
       </c>
       <c r="U139" s="5" t="s">
         <v>101</v>
@@ -14782,7 +14782,7 @@
         <v>100</v>
       </c>
       <c r="G154" s="22" t="n">
-        <v>2.65</v>
+        <v>2.95</v>
       </c>
       <c r="H154" s="6" t="n">
         <v>1170</v>
@@ -14833,7 +14833,7 @@
       </c>
       <c r="T154" s="23" t="n">
         <f aca="false">S154*G154*(1+Hypothèses!$B$22)</f>
-        <v>3.11779557320896</v>
+        <v>3.47075356262884</v>
       </c>
       <c r="U154" s="5" t="s">
         <v>101</v>
@@ -15995,7 +15995,7 @@
         <v>100</v>
       </c>
       <c r="G169" s="22" t="n">
-        <v>2.2</v>
+        <v>2.15</v>
       </c>
       <c r="H169" s="6" t="n">
         <v>1170</v>
@@ -16046,7 +16046,7 @@
       </c>
       <c r="T169" s="23" t="n">
         <f aca="false">S169*G169*(1+Hypothèses!$B$22)</f>
-        <v>2.58835858907914</v>
+        <v>2.52953225750916</v>
       </c>
       <c r="U169" s="5" t="s">
         <v>101</v>
@@ -17208,7 +17208,7 @@
         <v>100</v>
       </c>
       <c r="G184" s="22" t="n">
-        <v>2.6</v>
+        <v>2.85</v>
       </c>
       <c r="H184" s="6" t="n">
         <v>1170</v>
@@ -17259,7 +17259,7 @@
       </c>
       <c r="T184" s="23" t="n">
         <f aca="false">S184*G184*(1+Hypothèses!$B$22)</f>
-        <v>3.05896924163898</v>
+        <v>3.35310089948888</v>
       </c>
       <c r="U184" s="5" t="s">
         <v>101</v>
@@ -22176,9 +22176,11 @@
       <c r="E246" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="F246" s="21"/>
+      <c r="F246" s="21" t="s">
+        <v>387</v>
+      </c>
       <c r="G246" s="22" t="n">
-        <v>2.2</v>
+        <v>1.3</v>
       </c>
       <c r="H246" s="6" t="n">
         <v>6123</v>
@@ -22229,7 +22231,7 @@
       </c>
       <c r="T246" s="23" t="n">
         <f aca="false">S246*G246*(1+Hypothèses!$B$22)</f>
-        <v>1.92371484858461</v>
+        <v>1.13674059234545</v>
       </c>
       <c r="U246" s="5" t="s">
         <v>101</v>
@@ -22244,7 +22246,7 @@
         <v>27</v>
       </c>
       <c r="B247" s="21" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C247" s="21" t="s">
         <v>108</v>
@@ -22255,14 +22257,12 @@
       <c r="E247" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="F247" s="21" t="s">
-        <v>388</v>
-      </c>
+      <c r="F247" s="21"/>
       <c r="G247" s="22" t="n">
-        <v>1.3</v>
+        <v>2.3</v>
       </c>
       <c r="H247" s="6" t="n">
-        <v>6123</v>
+        <v>5991</v>
       </c>
       <c r="I247" s="23" t="n">
         <f aca="false">IF(A247="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H247,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H247,Hypothèses!$A$6:$A$16,1)))</f>
@@ -22270,7 +22270,7 @@
       </c>
       <c r="J247" s="24" t="n">
         <f aca="false">H247/3600/I247</f>
-        <v>0.283472222222222</v>
+        <v>0.277361111111111</v>
       </c>
       <c r="K247" s="21" t="n">
         <f aca="false">IF(A247="CTA 4",Hypothèses!$B$25,IF(AND(A247="CTA 5",H247&gt;4000),Hypothèses!$B$29,IF(H247&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -22278,15 +22278,15 @@
       </c>
       <c r="L247" s="21" t="n">
         <f aca="false">MAX(Hypothèses!$B$26,CEILING(J247/(K247/1000)*1000,Hypothèses!$B$27))</f>
-        <v>850</v>
+        <v>800</v>
       </c>
       <c r="M247" s="24" t="n">
         <f aca="false">L247*K247/1000000</f>
-        <v>0.2975</v>
+        <v>0.28</v>
       </c>
       <c r="N247" s="25" t="n">
         <f aca="false">H247/3600/M247</f>
-        <v>5.71708683473389</v>
+        <v>5.94345238095238</v>
       </c>
       <c r="O247" s="21" t="str">
         <f aca="false">IF(N247&lt;=I247,"oui","NON")</f>
@@ -22294,23 +22294,23 @@
       </c>
       <c r="P247" s="24" t="n">
         <f aca="false">1.3*((L247/1000)*(K247/1000))^0.625/((L247/1000)+(K247/1000))^0.25</f>
-        <v>0.582206965594154</v>
+        <v>0.566555763342023</v>
       </c>
       <c r="Q247" s="26" t="n">
         <f aca="false">N247*P247/Hypothèses!$B$20</f>
-        <v>221901.851872581</v>
+        <v>224486.480038496</v>
       </c>
       <c r="R247" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P247)+5.74/Q247^0.9))^2</f>
-        <v>0.0173062640953008</v>
+        <v>0.0173313373244756</v>
       </c>
       <c r="S247" s="25" t="n">
         <f aca="false">R247/P247*Hypothèses!$B$19*N247^2/2</f>
-        <v>0.582943893510489</v>
+        <v>0.648363023264328</v>
       </c>
       <c r="T247" s="23" t="n">
         <f aca="false">S247*G247*(1+Hypothèses!$B$22)</f>
-        <v>1.13674059234545</v>
+        <v>2.23685243026193</v>
       </c>
       <c r="U247" s="5" t="s">
         <v>101</v>
@@ -22340,10 +22340,10 @@
         <v>390</v>
       </c>
       <c r="G248" s="22" t="n">
-        <v>0.875</v>
+        <v>2.175</v>
       </c>
       <c r="H248" s="6" t="n">
-        <v>5994</v>
+        <v>5991</v>
       </c>
       <c r="I248" s="23" t="n">
         <f aca="false">IF(A248="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H248,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H248,Hypothèses!$A$6:$A$16,1)))</f>
@@ -22351,7 +22351,7 @@
       </c>
       <c r="J248" s="24" t="n">
         <f aca="false">H248/3600/I248</f>
-        <v>0.2775</v>
+        <v>0.277361111111111</v>
       </c>
       <c r="K248" s="21" t="n">
         <f aca="false">IF(A248="CTA 4",Hypothèses!$B$25,IF(AND(A248="CTA 5",H248&gt;4000),Hypothèses!$B$29,IF(H248&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -22367,7 +22367,7 @@
       </c>
       <c r="N248" s="25" t="n">
         <f aca="false">H248/3600/M248</f>
-        <v>5.94642857142857</v>
+        <v>5.94345238095238</v>
       </c>
       <c r="O248" s="21" t="str">
         <f aca="false">IF(N248&lt;=I248,"oui","NON")</f>
@@ -22379,19 +22379,19 @@
       </c>
       <c r="Q248" s="26" t="n">
         <f aca="false">N248*P248/Hypothèses!$B$20</f>
-        <v>224598.891896302</v>
+        <v>224486.480038496</v>
       </c>
       <c r="R248" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P248)+5.74/Q248^0.9))^2</f>
-        <v>0.0173303541791289</v>
+        <v>0.0173313373244756</v>
       </c>
       <c r="S248" s="25" t="n">
         <f aca="false">R248/P248*Hypothèses!$B$19*N248^2/2</f>
-        <v>0.648975706690844</v>
+        <v>0.648363023264328</v>
       </c>
       <c r="T248" s="23" t="n">
         <f aca="false">S248*G248*(1+Hypothèses!$B$22)</f>
-        <v>0.851780615031733</v>
+        <v>2.11528436339987</v>
       </c>
       <c r="U248" s="5" t="s">
         <v>101</v>
@@ -22418,13 +22418,13 @@
         <v>146</v>
       </c>
       <c r="F249" s="21" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="G249" s="22" t="n">
-        <v>1.198</v>
+        <v>3.025</v>
       </c>
       <c r="H249" s="6" t="n">
-        <v>5919</v>
+        <v>5916</v>
       </c>
       <c r="I249" s="23" t="n">
         <f aca="false">IF(A249="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H249,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H249,Hypothèses!$A$6:$A$16,1)))</f>
@@ -22432,7 +22432,7 @@
       </c>
       <c r="J249" s="24" t="n">
         <f aca="false">H249/3600/I249</f>
-        <v>0.274027777777778</v>
+        <v>0.273888888888889</v>
       </c>
       <c r="K249" s="21" t="n">
         <f aca="false">IF(A249="CTA 4",Hypothèses!$B$25,IF(AND(A249="CTA 5",H249&gt;4000),Hypothèses!$B$29,IF(H249&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -22448,7 +22448,7 @@
       </c>
       <c r="N249" s="25" t="n">
         <f aca="false">H249/3600/M249</f>
-        <v>5.87202380952381</v>
+        <v>5.86904761904762</v>
       </c>
       <c r="O249" s="21" t="str">
         <f aca="false">IF(N249&lt;=I249,"oui","NON")</f>
@@ -22460,19 +22460,19 @@
       </c>
       <c r="Q249" s="26" t="n">
         <f aca="false">N249*P249/Hypothèses!$B$20</f>
-        <v>221788.595451153</v>
+        <v>221676.183593347</v>
       </c>
       <c r="R249" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P249)+5.74/Q249^0.9))^2</f>
-        <v>0.0173551676945003</v>
+        <v>0.0173561705205719</v>
       </c>
       <c r="S249" s="25" t="n">
         <f aca="false">R249/P249*Hypothèses!$B$19*N249^2/2</f>
-        <v>0.633742771379918</v>
+        <v>0.633137100973236</v>
       </c>
       <c r="T249" s="23" t="n">
         <f aca="false">S249*G249*(1+Hypothèses!$B$22)</f>
-        <v>1.13883576016971</v>
+        <v>2.87285959566606</v>
       </c>
       <c r="U249" s="5" t="s">
         <v>101</v>
@@ -22499,13 +22499,13 @@
         <v>146</v>
       </c>
       <c r="F250" s="21" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="G250" s="22" t="n">
-        <v>1.827</v>
+        <v>3.188</v>
       </c>
       <c r="H250" s="6" t="n">
-        <v>5916</v>
+        <v>5808</v>
       </c>
       <c r="I250" s="23" t="n">
         <f aca="false">IF(A250="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H250,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H250,Hypothèses!$A$6:$A$16,1)))</f>
@@ -22513,7 +22513,7 @@
       </c>
       <c r="J250" s="24" t="n">
         <f aca="false">H250/3600/I250</f>
-        <v>0.273888888888889</v>
+        <v>0.268888888888889</v>
       </c>
       <c r="K250" s="21" t="n">
         <f aca="false">IF(A250="CTA 4",Hypothèses!$B$25,IF(AND(A250="CTA 5",H250&gt;4000),Hypothèses!$B$29,IF(H250&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -22529,7 +22529,7 @@
       </c>
       <c r="N250" s="25" t="n">
         <f aca="false">H250/3600/M250</f>
-        <v>5.86904761904762</v>
+        <v>5.76190476190476</v>
       </c>
       <c r="O250" s="21" t="str">
         <f aca="false">IF(N250&lt;=I250,"oui","NON")</f>
@@ -22541,19 +22541,19 @@
       </c>
       <c r="Q250" s="26" t="n">
         <f aca="false">N250*P250/Hypothèses!$B$20</f>
-        <v>221676.183593347</v>
+        <v>217629.356712333</v>
       </c>
       <c r="R250" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P250)+5.74/Q250^0.9))^2</f>
-        <v>0.0173561705205719</v>
+        <v>0.017392813186708</v>
       </c>
       <c r="S250" s="25" t="n">
         <f aca="false">R250/P250*Hypothèses!$B$19*N250^2/2</f>
-        <v>0.633137100973236</v>
+        <v>0.611519868577858</v>
       </c>
       <c r="T250" s="23" t="n">
         <f aca="false">S250*G250*(1+Hypothèses!$B$22)</f>
-        <v>1.73511222521715</v>
+        <v>2.92428801153932</v>
       </c>
       <c r="U250" s="5" t="s">
         <v>101</v>
@@ -22580,10 +22580,10 @@
         <v>146</v>
       </c>
       <c r="F251" s="21" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="G251" s="22" t="n">
-        <v>3.188</v>
+        <v>0.374</v>
       </c>
       <c r="H251" s="6" t="n">
         <v>5808</v>
@@ -22634,7 +22634,7 @@
       </c>
       <c r="T251" s="23" t="n">
         <f aca="false">S251*G251*(1+Hypothèses!$B$22)</f>
-        <v>2.92428801153932</v>
+        <v>0.343062646272178</v>
       </c>
       <c r="U251" s="5" t="s">
         <v>101</v>
@@ -22661,13 +22661,13 @@
         <v>146</v>
       </c>
       <c r="F252" s="21" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="G252" s="22" t="n">
-        <v>0.374</v>
+        <v>4.664</v>
       </c>
       <c r="H252" s="6" t="n">
-        <v>5808</v>
+        <v>5733</v>
       </c>
       <c r="I252" s="23" t="n">
         <f aca="false">IF(A252="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H252,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H252,Hypothèses!$A$6:$A$16,1)))</f>
@@ -22675,7 +22675,7 @@
       </c>
       <c r="J252" s="24" t="n">
         <f aca="false">H252/3600/I252</f>
-        <v>0.268888888888889</v>
+        <v>0.265416666666667</v>
       </c>
       <c r="K252" s="21" t="n">
         <f aca="false">IF(A252="CTA 4",Hypothèses!$B$25,IF(AND(A252="CTA 5",H252&gt;4000),Hypothèses!$B$29,IF(H252&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -22691,7 +22691,7 @@
       </c>
       <c r="N252" s="25" t="n">
         <f aca="false">H252/3600/M252</f>
-        <v>5.76190476190476</v>
+        <v>5.6875</v>
       </c>
       <c r="O252" s="21" t="str">
         <f aca="false">IF(N252&lt;=I252,"oui","NON")</f>
@@ -22703,19 +22703,19 @@
       </c>
       <c r="Q252" s="26" t="n">
         <f aca="false">N252*P252/Hypothèses!$B$20</f>
-        <v>217629.356712333</v>
+        <v>214819.060267184</v>
       </c>
       <c r="R252" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P252)+5.74/Q252^0.9))^2</f>
-        <v>0.017392813186708</v>
+        <v>0.0174188954385567</v>
       </c>
       <c r="S252" s="25" t="n">
         <f aca="false">R252/P252*Hypothèses!$B$19*N252^2/2</f>
-        <v>0.611519868577858</v>
+        <v>0.596721959276199</v>
       </c>
       <c r="T252" s="23" t="n">
         <f aca="false">S252*G252*(1+Hypothèses!$B$22)</f>
-        <v>0.343062646272178</v>
+        <v>4.17466682709629</v>
       </c>
       <c r="U252" s="5" t="s">
         <v>101</v>
@@ -22742,13 +22742,13 @@
         <v>146</v>
       </c>
       <c r="F253" s="21" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="G253" s="22" t="n">
-        <v>4.664</v>
+        <v>0.074</v>
       </c>
       <c r="H253" s="6" t="n">
-        <v>5733</v>
+        <v>5608</v>
       </c>
       <c r="I253" s="23" t="n">
         <f aca="false">IF(A253="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H253,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H253,Hypothèses!$A$6:$A$16,1)))</f>
@@ -22756,7 +22756,7 @@
       </c>
       <c r="J253" s="24" t="n">
         <f aca="false">H253/3600/I253</f>
-        <v>0.265416666666667</v>
+        <v>0.25962962962963</v>
       </c>
       <c r="K253" s="21" t="n">
         <f aca="false">IF(A253="CTA 4",Hypothèses!$B$25,IF(AND(A253="CTA 5",H253&gt;4000),Hypothèses!$B$29,IF(H253&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -22764,15 +22764,15 @@
       </c>
       <c r="L253" s="21" t="n">
         <f aca="false">MAX(Hypothèses!$B$26,CEILING(J253/(K253/1000)*1000,Hypothèses!$B$27))</f>
-        <v>800</v>
+        <v>750</v>
       </c>
       <c r="M253" s="24" t="n">
         <f aca="false">L253*K253/1000000</f>
-        <v>0.28</v>
+        <v>0.2625</v>
       </c>
       <c r="N253" s="25" t="n">
         <f aca="false">H253/3600/M253</f>
-        <v>5.6875</v>
+        <v>5.93439153439153</v>
       </c>
       <c r="O253" s="21" t="str">
         <f aca="false">IF(N253&lt;=I253,"oui","NON")</f>
@@ -22780,23 +22780,23 @@
       </c>
       <c r="P253" s="24" t="n">
         <f aca="false">1.3*((L253/1000)*(K253/1000))^0.625/((L253/1000)+(K253/1000))^0.25</f>
-        <v>0.566555763342023</v>
+        <v>0.550238530157161</v>
       </c>
       <c r="Q253" s="26" t="n">
         <f aca="false">N253*P253/Hypothèses!$B$20</f>
-        <v>214819.060267184</v>
+        <v>217688.72501738</v>
       </c>
       <c r="R253" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P253)+5.74/Q253^0.9))^2</f>
-        <v>0.0174188954385567</v>
+        <v>0.0174443385643649</v>
       </c>
       <c r="S253" s="25" t="n">
         <f aca="false">R253/P253*Hypothèses!$B$19*N253^2/2</f>
-        <v>0.596721959276199</v>
+        <v>0.669895641091274</v>
       </c>
       <c r="T253" s="23" t="n">
         <f aca="false">S253*G253*(1+Hypothèses!$B$22)</f>
-        <v>4.17466682709629</v>
+        <v>0.0743584161611315</v>
       </c>
       <c r="U253" s="5" t="s">
         <v>101</v>
@@ -22822,14 +22822,12 @@
       <c r="E254" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="F254" s="21" t="s">
-        <v>325</v>
-      </c>
+      <c r="F254" s="21"/>
       <c r="G254" s="22" t="n">
-        <v>0.074</v>
+        <v>6.15</v>
       </c>
       <c r="H254" s="6" t="n">
-        <v>5608</v>
+        <v>5374</v>
       </c>
       <c r="I254" s="23" t="n">
         <f aca="false">IF(A254="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H254,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H254,Hypothèses!$A$6:$A$16,1)))</f>
@@ -22837,7 +22835,7 @@
       </c>
       <c r="J254" s="24" t="n">
         <f aca="false">H254/3600/I254</f>
-        <v>0.25962962962963</v>
+        <v>0.248796296296296</v>
       </c>
       <c r="K254" s="21" t="n">
         <f aca="false">IF(A254="CTA 4",Hypothèses!$B$25,IF(AND(A254="CTA 5",H254&gt;4000),Hypothèses!$B$29,IF(H254&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -22853,7 +22851,7 @@
       </c>
       <c r="N254" s="25" t="n">
         <f aca="false">H254/3600/M254</f>
-        <v>5.93439153439153</v>
+        <v>5.68677248677249</v>
       </c>
       <c r="O254" s="21" t="str">
         <f aca="false">IF(N254&lt;=I254,"oui","NON")</f>
@@ -22865,19 +22863,19 @@
       </c>
       <c r="Q254" s="26" t="n">
         <f aca="false">N254*P254/Hypothèses!$B$20</f>
-        <v>217688.72501738</v>
+        <v>208605.422297325</v>
       </c>
       <c r="R254" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P254)+5.74/Q254^0.9))^2</f>
-        <v>0.0174443385643649</v>
+        <v>0.0175298544810203</v>
       </c>
       <c r="S254" s="25" t="n">
         <f aca="false">R254/P254*Hypothèses!$B$19*N254^2/2</f>
-        <v>0.669895641091274</v>
+        <v>0.618173338373011</v>
       </c>
       <c r="T254" s="23" t="n">
         <f aca="false">S254*G254*(1+Hypothèses!$B$22)</f>
-        <v>0.0743584161611315</v>
+        <v>5.70264904649103</v>
       </c>
       <c r="U254" s="5" t="s">
         <v>101</v>
@@ -22903,11 +22901,9 @@
       <c r="E255" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="F255" s="21" t="s">
-        <v>327</v>
-      </c>
+      <c r="F255" s="21"/>
       <c r="G255" s="22" t="n">
-        <v>3.712</v>
+        <v>1.4</v>
       </c>
       <c r="H255" s="6" t="n">
         <v>5374</v>
@@ -22958,7 +22954,7 @@
       </c>
       <c r="T255" s="23" t="n">
         <f aca="false">S255*G255*(1+Hypothèses!$B$22)</f>
-        <v>3.44198914806093</v>
+        <v>1.29816401058332</v>
       </c>
       <c r="U255" s="5" t="s">
         <v>101</v>
@@ -22985,10 +22981,10 @@
         <v>146</v>
       </c>
       <c r="F256" s="21" t="s">
-        <v>329</v>
+        <v>399</v>
       </c>
       <c r="G256" s="22" t="n">
-        <v>0.172</v>
+        <v>1.3</v>
       </c>
       <c r="H256" s="6" t="n">
         <v>5374</v>
@@ -23039,7 +23035,7 @@
       </c>
       <c r="T256" s="23" t="n">
         <f aca="false">S256*G256*(1+Hypothèses!$B$22)</f>
-        <v>0.159488721300237</v>
+        <v>1.20543800982737</v>
       </c>
       <c r="U256" s="5" t="s">
         <v>101</v>
@@ -23054,7 +23050,7 @@
         <v>27</v>
       </c>
       <c r="B257" s="21" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C257" s="21" t="s">
         <v>108</v>
@@ -23066,13 +23062,13 @@
         <v>146</v>
       </c>
       <c r="F257" s="21" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="G257" s="22" t="n">
-        <v>1.765</v>
+        <v>0.474</v>
       </c>
       <c r="H257" s="6" t="n">
-        <v>5249</v>
+        <v>5149</v>
       </c>
       <c r="I257" s="23" t="n">
         <f aca="false">IF(A257="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H257,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H257,Hypothèses!$A$6:$A$16,1)))</f>
@@ -23080,7 +23076,7 @@
       </c>
       <c r="J257" s="24" t="n">
         <f aca="false">H257/3600/I257</f>
-        <v>0.243009259259259</v>
+        <v>0.23837962962963</v>
       </c>
       <c r="K257" s="21" t="n">
         <f aca="false">IF(A257="CTA 4",Hypothèses!$B$25,IF(AND(A257="CTA 5",H257&gt;4000),Hypothèses!$B$29,IF(H257&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -23096,7 +23092,7 @@
       </c>
       <c r="N257" s="25" t="n">
         <f aca="false">H257/3600/M257</f>
-        <v>5.95124716553288</v>
+        <v>5.83786848072562</v>
       </c>
       <c r="O257" s="21" t="str">
         <f aca="false">IF(N257&lt;=I257,"oui","NON")</f>
@@ -23108,19 +23104,19 @@
       </c>
       <c r="Q257" s="26" t="n">
         <f aca="false">N257*P257/Hypothèses!$B$20</f>
-        <v>211539.541567357</v>
+        <v>207509.449329457</v>
       </c>
       <c r="R257" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P257)+5.74/Q257^0.9))^2</f>
-        <v>0.0175583939769815</v>
+        <v>0.017597006572538</v>
       </c>
       <c r="S257" s="25" t="n">
         <f aca="false">R257/P257*Hypothèses!$B$19*N257^2/2</f>
-        <v>0.699805231720433</v>
+        <v>0.67487576031149</v>
       </c>
       <c r="T257" s="23" t="n">
         <f aca="false">S257*G257*(1+Hypothèses!$B$22)</f>
-        <v>1.85273435097985</v>
+        <v>0.47983666558147</v>
       </c>
       <c r="U257" s="5" t="s">
         <v>101</v>
@@ -23135,7 +23131,7 @@
         <v>27</v>
       </c>
       <c r="B258" s="21" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C258" s="21" t="s">
         <v>108</v>
@@ -23146,14 +23142,12 @@
       <c r="E258" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="F258" s="21" t="s">
-        <v>333</v>
-      </c>
+      <c r="F258" s="21"/>
       <c r="G258" s="22" t="n">
-        <v>2.275</v>
+        <v>4.476</v>
       </c>
       <c r="H258" s="6" t="n">
-        <v>5249</v>
+        <v>5149</v>
       </c>
       <c r="I258" s="23" t="n">
         <f aca="false">IF(A258="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H258,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H258,Hypothèses!$A$6:$A$16,1)))</f>
@@ -23161,7 +23155,7 @@
       </c>
       <c r="J258" s="24" t="n">
         <f aca="false">H258/3600/I258</f>
-        <v>0.243009259259259</v>
+        <v>0.23837962962963</v>
       </c>
       <c r="K258" s="21" t="n">
         <f aca="false">IF(A258="CTA 4",Hypothèses!$B$25,IF(AND(A258="CTA 5",H258&gt;4000),Hypothèses!$B$29,IF(H258&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -23177,7 +23171,7 @@
       </c>
       <c r="N258" s="25" t="n">
         <f aca="false">H258/3600/M258</f>
-        <v>5.95124716553288</v>
+        <v>5.83786848072562</v>
       </c>
       <c r="O258" s="21" t="str">
         <f aca="false">IF(N258&lt;=I258,"oui","NON")</f>
@@ -23189,19 +23183,19 @@
       </c>
       <c r="Q258" s="26" t="n">
         <f aca="false">N258*P258/Hypothèses!$B$20</f>
-        <v>211539.541567357</v>
+        <v>207509.449329457</v>
       </c>
       <c r="R258" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P258)+5.74/Q258^0.9))^2</f>
-        <v>0.0175583939769815</v>
+        <v>0.017597006572538</v>
       </c>
       <c r="S258" s="25" t="n">
         <f aca="false">R258/P258*Hypothèses!$B$19*N258^2/2</f>
-        <v>0.699805231720433</v>
+        <v>0.67487576031149</v>
       </c>
       <c r="T258" s="23" t="n">
         <f aca="false">S258*G258*(1+Hypothèses!$B$22)</f>
-        <v>2.38808535324598</v>
+        <v>4.53111585473135</v>
       </c>
       <c r="U258" s="5" t="s">
         <v>101</v>
@@ -23216,7 +23210,7 @@
         <v>27</v>
       </c>
       <c r="B259" s="21" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C259" s="21" t="s">
         <v>108</v>
@@ -23227,12 +23221,14 @@
       <c r="E259" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="F259" s="21"/>
+      <c r="F259" s="21" t="s">
+        <v>344</v>
+      </c>
       <c r="G259" s="22" t="n">
-        <v>4.476</v>
+        <v>1.3</v>
       </c>
       <c r="H259" s="6" t="n">
-        <v>5149</v>
+        <v>5147</v>
       </c>
       <c r="I259" s="23" t="n">
         <f aca="false">IF(A259="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H259,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H259,Hypothèses!$A$6:$A$16,1)))</f>
@@ -23240,7 +23236,7 @@
       </c>
       <c r="J259" s="24" t="n">
         <f aca="false">H259/3600/I259</f>
-        <v>0.23837962962963</v>
+        <v>0.238287037037037</v>
       </c>
       <c r="K259" s="21" t="n">
         <f aca="false">IF(A259="CTA 4",Hypothèses!$B$25,IF(AND(A259="CTA 5",H259&gt;4000),Hypothèses!$B$29,IF(H259&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -23256,7 +23252,7 @@
       </c>
       <c r="N259" s="25" t="n">
         <f aca="false">H259/3600/M259</f>
-        <v>5.83786848072562</v>
+        <v>5.83560090702948</v>
       </c>
       <c r="O259" s="21" t="str">
         <f aca="false">IF(N259&lt;=I259,"oui","NON")</f>
@@ -23268,19 +23264,19 @@
       </c>
       <c r="Q259" s="26" t="n">
         <f aca="false">N259*P259/Hypothèses!$B$20</f>
-        <v>207509.449329457</v>
+        <v>207428.847484699</v>
       </c>
       <c r="R259" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P259)+5.74/Q259^0.9))^2</f>
-        <v>0.017597006572538</v>
+        <v>0.0175977908596456</v>
       </c>
       <c r="S259" s="25" t="n">
         <f aca="false">R259/P259*Hypothèses!$B$19*N259^2/2</f>
-        <v>0.67487576031149</v>
+        <v>0.674381640393831</v>
       </c>
       <c r="T259" s="23" t="n">
         <f aca="false">S259*G259*(1+Hypothèses!$B$22)</f>
-        <v>4.53111585473135</v>
+        <v>1.31504419876797</v>
       </c>
       <c r="U259" s="5" t="s">
         <v>101</v>
@@ -23295,7 +23291,7 @@
         <v>27</v>
       </c>
       <c r="B260" s="21" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C260" s="21" t="s">
         <v>108</v>
@@ -23307,13 +23303,13 @@
         <v>146</v>
       </c>
       <c r="F260" s="21" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="G260" s="22" t="n">
-        <v>1.3</v>
+        <v>0.9</v>
       </c>
       <c r="H260" s="6" t="n">
-        <v>5147</v>
+        <v>5143</v>
       </c>
       <c r="I260" s="23" t="n">
         <f aca="false">IF(A260="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H260,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H260,Hypothèses!$A$6:$A$16,1)))</f>
@@ -23321,7 +23317,7 @@
       </c>
       <c r="J260" s="24" t="n">
         <f aca="false">H260/3600/I260</f>
-        <v>0.238287037037037</v>
+        <v>0.238101851851852</v>
       </c>
       <c r="K260" s="21" t="n">
         <f aca="false">IF(A260="CTA 4",Hypothèses!$B$25,IF(AND(A260="CTA 5",H260&gt;4000),Hypothèses!$B$29,IF(H260&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -23337,7 +23333,7 @@
       </c>
       <c r="N260" s="25" t="n">
         <f aca="false">H260/3600/M260</f>
-        <v>5.83560090702948</v>
+        <v>5.83106575963719</v>
       </c>
       <c r="O260" s="21" t="str">
         <f aca="false">IF(N260&lt;=I260,"oui","NON")</f>
@@ -23349,19 +23345,19 @@
       </c>
       <c r="Q260" s="26" t="n">
         <f aca="false">N260*P260/Hypothèses!$B$20</f>
-        <v>207428.847484699</v>
+        <v>207267.643795183</v>
       </c>
       <c r="R260" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P260)+5.74/Q260^0.9))^2</f>
-        <v>0.0175977908596456</v>
+        <v>0.0175993608740412</v>
       </c>
       <c r="S260" s="25" t="n">
         <f aca="false">R260/P260*Hypothèses!$B$19*N260^2/2</f>
-        <v>0.674381640393831</v>
+        <v>0.673393926499009</v>
       </c>
       <c r="T260" s="23" t="n">
         <f aca="false">S260*G260*(1+Hypothèses!$B$22)</f>
-        <v>1.31504419876797</v>
+        <v>0.909081800773662</v>
       </c>
       <c r="U260" s="5" t="s">
         <v>101</v>
@@ -23376,7 +23372,7 @@
         <v>27</v>
       </c>
       <c r="B261" s="21" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C261" s="21" t="s">
         <v>108</v>
@@ -23387,38 +23383,36 @@
       <c r="E261" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="F261" s="21" t="s">
-        <v>336</v>
-      </c>
+      <c r="F261" s="21"/>
       <c r="G261" s="22" t="n">
-        <v>0.9</v>
+        <v>2.9</v>
       </c>
       <c r="H261" s="6" t="n">
-        <v>5143</v>
+        <v>3113</v>
       </c>
       <c r="I261" s="23" t="n">
         <f aca="false">IF(A261="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H261,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H261,Hypothèses!$A$6:$A$16,1)))</f>
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="J261" s="24" t="n">
         <f aca="false">H261/3600/I261</f>
-        <v>0.238101851851852</v>
+        <v>0.157222222222222</v>
       </c>
       <c r="K261" s="21" t="n">
         <f aca="false">IF(A261="CTA 4",Hypothèses!$B$25,IF(AND(A261="CTA 5",H261&gt;4000),Hypothèses!$B$29,IF(H261&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
-        <v>350</v>
+        <v>300</v>
       </c>
       <c r="L261" s="21" t="n">
         <f aca="false">MAX(Hypothèses!$B$26,CEILING(J261/(K261/1000)*1000,Hypothèses!$B$27))</f>
-        <v>700</v>
+        <v>550</v>
       </c>
       <c r="M261" s="24" t="n">
         <f aca="false">L261*K261/1000000</f>
-        <v>0.245</v>
+        <v>0.165</v>
       </c>
       <c r="N261" s="25" t="n">
         <f aca="false">H261/3600/M261</f>
-        <v>5.83106575963719</v>
+        <v>5.24074074074074</v>
       </c>
       <c r="O261" s="21" t="str">
         <f aca="false">IF(N261&lt;=I261,"oui","NON")</f>
@@ -23426,23 +23420,23 @@
       </c>
       <c r="P261" s="24" t="n">
         <f aca="false">1.3*((L261/1000)*(K261/1000))^0.625/((L261/1000)+(K261/1000))^0.25</f>
-        <v>0.533181203074134</v>
+        <v>0.439052127572127</v>
       </c>
       <c r="Q261" s="26" t="n">
         <f aca="false">N261*P261/Hypothèses!$B$20</f>
-        <v>207267.643795183</v>
+        <v>153397.22481841</v>
       </c>
       <c r="R261" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P261)+5.74/Q261^0.9))^2</f>
-        <v>0.0175993608740412</v>
+        <v>0.0186031259838118</v>
       </c>
       <c r="S261" s="25" t="n">
         <f aca="false">R261/P261*Hypothèses!$B$19*N261^2/2</f>
-        <v>0.673393926499009</v>
+        <v>0.69824276277717</v>
       </c>
       <c r="T261" s="23" t="n">
         <f aca="false">S261*G261*(1+Hypothèses!$B$22)</f>
-        <v>0.909081800773662</v>
+        <v>3.03735601808069</v>
       </c>
       <c r="U261" s="5" t="s">
         <v>101</v>
@@ -23457,7 +23451,7 @@
         <v>27</v>
       </c>
       <c r="B262" s="21" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C262" s="21" t="s">
         <v>108</v>
@@ -23468,9 +23462,11 @@
       <c r="E262" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="F262" s="21"/>
+      <c r="F262" s="21" t="s">
+        <v>406</v>
+      </c>
       <c r="G262" s="22" t="n">
-        <v>2.9</v>
+        <v>1.3</v>
       </c>
       <c r="H262" s="6" t="n">
         <v>3113</v>
@@ -23521,7 +23517,7 @@
       </c>
       <c r="T262" s="23" t="n">
         <f aca="false">S262*G262*(1+Hypothèses!$B$22)</f>
-        <v>3.03735601808069</v>
+        <v>1.36157338741548</v>
       </c>
       <c r="U262" s="5" t="s">
         <v>101</v>
@@ -23536,7 +23532,7 @@
         <v>27</v>
       </c>
       <c r="B263" s="21" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="C263" s="21" t="s">
         <v>108</v>
@@ -23547,14 +23543,12 @@
       <c r="E263" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="F263" s="21" t="s">
-        <v>406</v>
-      </c>
+      <c r="F263" s="21"/>
       <c r="G263" s="22" t="n">
-        <v>1.3</v>
+        <v>2.23</v>
       </c>
       <c r="H263" s="6" t="n">
-        <v>3113</v>
+        <v>3061</v>
       </c>
       <c r="I263" s="23" t="n">
         <f aca="false">IF(A263="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H263,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H263,Hypothèses!$A$6:$A$16,1)))</f>
@@ -23562,7 +23556,7 @@
       </c>
       <c r="J263" s="24" t="n">
         <f aca="false">H263/3600/I263</f>
-        <v>0.157222222222222</v>
+        <v>0.15459595959596</v>
       </c>
       <c r="K263" s="21" t="n">
         <f aca="false">IF(A263="CTA 4",Hypothèses!$B$25,IF(AND(A263="CTA 5",H263&gt;4000),Hypothèses!$B$29,IF(H263&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -23578,7 +23572,7 @@
       </c>
       <c r="N263" s="25" t="n">
         <f aca="false">H263/3600/M263</f>
-        <v>5.24074074074074</v>
+        <v>5.15319865319865</v>
       </c>
       <c r="O263" s="21" t="str">
         <f aca="false">IF(N263&lt;=I263,"oui","NON")</f>
@@ -23590,19 +23584,19 @@
       </c>
       <c r="Q263" s="26" t="n">
         <f aca="false">N263*P263/Hypothèses!$B$20</f>
-        <v>153397.22481841</v>
+        <v>150834.855499246</v>
       </c>
       <c r="R263" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P263)+5.74/Q263^0.9))^2</f>
-        <v>0.0186031259838118</v>
+        <v>0.0186415467296234</v>
       </c>
       <c r="S263" s="25" t="n">
         <f aca="false">R263/P263*Hypothèses!$B$19*N263^2/2</f>
-        <v>0.69824276277717</v>
+        <v>0.676504792339363</v>
       </c>
       <c r="T263" s="23" t="n">
         <f aca="false">S263*G263*(1+Hypothèses!$B$22)</f>
-        <v>1.36157338741548</v>
+        <v>2.26290853037517</v>
       </c>
       <c r="U263" s="5" t="s">
         <v>101</v>
@@ -23617,7 +23611,7 @@
         <v>27</v>
       </c>
       <c r="B264" s="21" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C264" s="21" t="s">
         <v>108</v>
@@ -23628,9 +23622,11 @@
       <c r="E264" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="F264" s="21"/>
+      <c r="F264" s="21" t="s">
+        <v>409</v>
+      </c>
       <c r="G264" s="22" t="n">
-        <v>2.23</v>
+        <v>1.3</v>
       </c>
       <c r="H264" s="6" t="n">
         <v>3061</v>
@@ -23681,7 +23677,7 @@
       </c>
       <c r="T264" s="23" t="n">
         <f aca="false">S264*G264*(1+Hypothèses!$B$22)</f>
-        <v>2.26290853037517</v>
+        <v>1.31918434506176</v>
       </c>
       <c r="U264" s="5" t="s">
         <v>101</v>
@@ -23696,7 +23692,7 @@
         <v>27</v>
       </c>
       <c r="B265" s="21" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="C265" s="21" t="s">
         <v>108</v>
@@ -23707,14 +23703,12 @@
       <c r="E265" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="F265" s="21" t="s">
-        <v>409</v>
-      </c>
+      <c r="F265" s="21"/>
       <c r="G265" s="22" t="n">
-        <v>1.3</v>
+        <v>3.88</v>
       </c>
       <c r="H265" s="6" t="n">
-        <v>3061</v>
+        <v>2852</v>
       </c>
       <c r="I265" s="23" t="n">
         <f aca="false">IF(A265="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H265,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H265,Hypothèses!$A$6:$A$16,1)))</f>
@@ -23722,7 +23716,7 @@
       </c>
       <c r="J265" s="24" t="n">
         <f aca="false">H265/3600/I265</f>
-        <v>0.15459595959596</v>
+        <v>0.144040404040404</v>
       </c>
       <c r="K265" s="21" t="n">
         <f aca="false">IF(A265="CTA 4",Hypothèses!$B$25,IF(AND(A265="CTA 5",H265&gt;4000),Hypothèses!$B$29,IF(H265&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -23730,15 +23724,15 @@
       </c>
       <c r="L265" s="21" t="n">
         <f aca="false">MAX(Hypothèses!$B$26,CEILING(J265/(K265/1000)*1000,Hypothèses!$B$27))</f>
-        <v>550</v>
+        <v>500</v>
       </c>
       <c r="M265" s="24" t="n">
         <f aca="false">L265*K265/1000000</f>
-        <v>0.165</v>
+        <v>0.15</v>
       </c>
       <c r="N265" s="25" t="n">
         <f aca="false">H265/3600/M265</f>
-        <v>5.15319865319865</v>
+        <v>5.28148148148148</v>
       </c>
       <c r="O265" s="21" t="str">
         <f aca="false">IF(N265&lt;=I265,"oui","NON")</f>
@@ -23746,23 +23740,23 @@
       </c>
       <c r="P265" s="24" t="n">
         <f aca="false">1.3*((L265/1000)*(K265/1000))^0.625/((L265/1000)+(K265/1000))^0.25</f>
-        <v>0.439052127572127</v>
+        <v>0.419979306877563</v>
       </c>
       <c r="Q265" s="26" t="n">
         <f aca="false">N265*P265/Hypothèses!$B$20</f>
-        <v>150834.855499246</v>
+        <v>147874.195458619</v>
       </c>
       <c r="R265" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P265)+5.74/Q265^0.9))^2</f>
-        <v>0.0186415467296234</v>
+        <v>0.0187713117156423</v>
       </c>
       <c r="S265" s="25" t="n">
         <f aca="false">R265/P265*Hypothèses!$B$19*N265^2/2</f>
-        <v>0.676504792339363</v>
+        <v>0.748048062227502</v>
       </c>
       <c r="T265" s="23" t="n">
         <f aca="false">S265*G265*(1+Hypothèses!$B$22)</f>
-        <v>1.31918434506176</v>
+        <v>4.35363972216406</v>
       </c>
       <c r="U265" s="5" t="s">
         <v>101</v>
@@ -23777,7 +23771,7 @@
         <v>27</v>
       </c>
       <c r="B266" s="21" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C266" s="21" t="s">
         <v>108</v>
@@ -23788,9 +23782,11 @@
       <c r="E266" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="F266" s="21"/>
+      <c r="F266" s="21" t="s">
+        <v>346</v>
+      </c>
       <c r="G266" s="22" t="n">
-        <v>3.88</v>
+        <v>3.251</v>
       </c>
       <c r="H266" s="6" t="n">
         <v>2852</v>
@@ -23841,7 +23837,7 @@
       </c>
       <c r="T266" s="23" t="n">
         <f aca="false">S266*G266*(1+Hypothèses!$B$22)</f>
-        <v>4.35363972216406</v>
+        <v>3.64785637545241</v>
       </c>
       <c r="U266" s="5" t="s">
         <v>101</v>
@@ -23856,7 +23852,7 @@
         <v>27</v>
       </c>
       <c r="B267" s="21" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C267" s="21" t="s">
         <v>108</v>
@@ -23868,13 +23864,13 @@
         <v>146</v>
       </c>
       <c r="F267" s="21" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="G267" s="22" t="n">
-        <v>3.251</v>
+        <v>1.602</v>
       </c>
       <c r="H267" s="6" t="n">
-        <v>2852</v>
+        <v>2847</v>
       </c>
       <c r="I267" s="23" t="n">
         <f aca="false">IF(A267="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H267,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H267,Hypothèses!$A$6:$A$16,1)))</f>
@@ -23882,7 +23878,7 @@
       </c>
       <c r="J267" s="24" t="n">
         <f aca="false">H267/3600/I267</f>
-        <v>0.144040404040404</v>
+        <v>0.143787878787879</v>
       </c>
       <c r="K267" s="21" t="n">
         <f aca="false">IF(A267="CTA 4",Hypothèses!$B$25,IF(AND(A267="CTA 5",H267&gt;4000),Hypothèses!$B$29,IF(H267&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -23898,7 +23894,7 @@
       </c>
       <c r="N267" s="25" t="n">
         <f aca="false">H267/3600/M267</f>
-        <v>5.28148148148148</v>
+        <v>5.27222222222222</v>
       </c>
       <c r="O267" s="21" t="str">
         <f aca="false">IF(N267&lt;=I267,"oui","NON")</f>
@@ -23910,19 +23906,19 @@
       </c>
       <c r="Q267" s="26" t="n">
         <f aca="false">N267*P267/Hypothèses!$B$20</f>
-        <v>147874.195458619</v>
+        <v>147614.948972892</v>
       </c>
       <c r="R267" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P267)+5.74/Q267^0.9))^2</f>
-        <v>0.0187713117156423</v>
+        <v>0.0187753311653781</v>
       </c>
       <c r="S267" s="25" t="n">
         <f aca="false">R267/P267*Hypothèses!$B$19*N267^2/2</f>
-        <v>0.748048062227502</v>
+        <v>0.745587088325204</v>
       </c>
       <c r="T267" s="23" t="n">
         <f aca="false">S267*G267*(1+Hypothèses!$B$22)</f>
-        <v>3.64785637545241</v>
+        <v>1.79164577324547</v>
       </c>
       <c r="U267" s="5" t="s">
         <v>101</v>
@@ -23937,7 +23933,7 @@
         <v>27</v>
       </c>
       <c r="B268" s="21" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C268" s="21" t="s">
         <v>108</v>
@@ -23949,10 +23945,10 @@
         <v>146</v>
       </c>
       <c r="F268" s="21" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="G268" s="22" t="n">
-        <v>1.602</v>
+        <v>2.352</v>
       </c>
       <c r="H268" s="6" t="n">
         <v>2847</v>
@@ -24003,7 +23999,7 @@
       </c>
       <c r="T268" s="23" t="n">
         <f aca="false">S268*G268*(1+Hypothèses!$B$22)</f>
-        <v>1.79164577324547</v>
+        <v>2.63043124761132</v>
       </c>
       <c r="U268" s="5" t="s">
         <v>101</v>
@@ -24018,7 +24014,7 @@
         <v>27</v>
       </c>
       <c r="B269" s="21" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C269" s="21" t="s">
         <v>108</v>
@@ -24030,13 +24026,13 @@
         <v>146</v>
       </c>
       <c r="F269" s="21" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="G269" s="22" t="n">
-        <v>2.352</v>
+        <v>2.268</v>
       </c>
       <c r="H269" s="6" t="n">
-        <v>2847</v>
+        <v>2752</v>
       </c>
       <c r="I269" s="23" t="n">
         <f aca="false">IF(A269="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H269,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H269,Hypothèses!$A$6:$A$16,1)))</f>
@@ -24044,7 +24040,7 @@
       </c>
       <c r="J269" s="24" t="n">
         <f aca="false">H269/3600/I269</f>
-        <v>0.143787878787879</v>
+        <v>0.138989898989899</v>
       </c>
       <c r="K269" s="21" t="n">
         <f aca="false">IF(A269="CTA 4",Hypothèses!$B$25,IF(AND(A269="CTA 5",H269&gt;4000),Hypothèses!$B$29,IF(H269&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -24060,7 +24056,7 @@
       </c>
       <c r="N269" s="25" t="n">
         <f aca="false">H269/3600/M269</f>
-        <v>5.27222222222222</v>
+        <v>5.0962962962963</v>
       </c>
       <c r="O269" s="21" t="str">
         <f aca="false">IF(N269&lt;=I269,"oui","NON")</f>
@@ -24072,19 +24068,19 @@
       </c>
       <c r="Q269" s="26" t="n">
         <f aca="false">N269*P269/Hypothèses!$B$20</f>
-        <v>147614.948972892</v>
+        <v>142689.265744081</v>
       </c>
       <c r="R269" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P269)+5.74/Q269^0.9))^2</f>
-        <v>0.0187753311653781</v>
+        <v>0.0188538668550145</v>
       </c>
       <c r="S269" s="25" t="n">
         <f aca="false">R269/P269*Hypothèses!$B$19*N269^2/2</f>
-        <v>0.745587088325204</v>
+        <v>0.699573150839758</v>
       </c>
       <c r="T269" s="23" t="n">
         <f aca="false">S269*G269*(1+Hypothèses!$B$22)</f>
-        <v>2.63043124761132</v>
+        <v>2.37994785915686</v>
       </c>
       <c r="U269" s="5" t="s">
         <v>101</v>
@@ -24099,7 +24095,7 @@
         <v>27</v>
       </c>
       <c r="B270" s="21" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C270" s="21" t="s">
         <v>108</v>
@@ -24111,13 +24107,13 @@
         <v>146</v>
       </c>
       <c r="F270" s="21" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="G270" s="22" t="n">
-        <v>2.268</v>
+        <v>0.498</v>
       </c>
       <c r="H270" s="6" t="n">
-        <v>2752</v>
+        <v>2748</v>
       </c>
       <c r="I270" s="23" t="n">
         <f aca="false">IF(A270="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H270,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H270,Hypothèses!$A$6:$A$16,1)))</f>
@@ -24125,7 +24121,7 @@
       </c>
       <c r="J270" s="24" t="n">
         <f aca="false">H270/3600/I270</f>
-        <v>0.138989898989899</v>
+        <v>0.138787878787879</v>
       </c>
       <c r="K270" s="21" t="n">
         <f aca="false">IF(A270="CTA 4",Hypothèses!$B$25,IF(AND(A270="CTA 5",H270&gt;4000),Hypothèses!$B$29,IF(H270&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -24141,7 +24137,7 @@
       </c>
       <c r="N270" s="25" t="n">
         <f aca="false">H270/3600/M270</f>
-        <v>5.0962962962963</v>
+        <v>5.08888888888889</v>
       </c>
       <c r="O270" s="21" t="str">
         <f aca="false">IF(N270&lt;=I270,"oui","NON")</f>
@@ -24153,19 +24149,19 @@
       </c>
       <c r="Q270" s="26" t="n">
         <f aca="false">N270*P270/Hypothèses!$B$20</f>
-        <v>142689.265744081</v>
+        <v>142481.868555499</v>
       </c>
       <c r="R270" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P270)+5.74/Q270^0.9))^2</f>
-        <v>0.0188538668550145</v>
+        <v>0.0188572667473426</v>
       </c>
       <c r="S270" s="25" t="n">
         <f aca="false">R270/P270*Hypothèses!$B$19*N270^2/2</f>
-        <v>0.699573150839758</v>
+        <v>0.697666772520778</v>
       </c>
       <c r="T270" s="23" t="n">
         <f aca="false">S270*G270*(1+Hypothèses!$B$22)</f>
-        <v>2.37994785915686</v>
+        <v>0.521157079073021</v>
       </c>
       <c r="U270" s="5" t="s">
         <v>101</v>
@@ -24180,7 +24176,7 @@
         <v>27</v>
       </c>
       <c r="B271" s="21" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C271" s="21" t="s">
         <v>108</v>
@@ -24192,13 +24188,13 @@
         <v>146</v>
       </c>
       <c r="F271" s="21" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="G271" s="22" t="n">
-        <v>0.498</v>
+        <v>0.264</v>
       </c>
       <c r="H271" s="6" t="n">
-        <v>2748</v>
+        <v>2727</v>
       </c>
       <c r="I271" s="23" t="n">
         <f aca="false">IF(A271="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H271,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H271,Hypothèses!$A$6:$A$16,1)))</f>
@@ -24206,7 +24202,7 @@
       </c>
       <c r="J271" s="24" t="n">
         <f aca="false">H271/3600/I271</f>
-        <v>0.138787878787879</v>
+        <v>0.137727272727273</v>
       </c>
       <c r="K271" s="21" t="n">
         <f aca="false">IF(A271="CTA 4",Hypothèses!$B$25,IF(AND(A271="CTA 5",H271&gt;4000),Hypothèses!$B$29,IF(H271&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -24222,7 +24218,7 @@
       </c>
       <c r="N271" s="25" t="n">
         <f aca="false">H271/3600/M271</f>
-        <v>5.08888888888889</v>
+        <v>5.05</v>
       </c>
       <c r="O271" s="21" t="str">
         <f aca="false">IF(N271&lt;=I271,"oui","NON")</f>
@@ -24234,19 +24230,19 @@
       </c>
       <c r="Q271" s="26" t="n">
         <f aca="false">N271*P271/Hypothèses!$B$20</f>
-        <v>142481.868555499</v>
+        <v>141393.033315446</v>
       </c>
       <c r="R271" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P271)+5.74/Q271^0.9))^2</f>
-        <v>0.0188572667473426</v>
+        <v>0.018875244148939</v>
       </c>
       <c r="S271" s="25" t="n">
         <f aca="false">R271/P271*Hypothèses!$B$19*N271^2/2</f>
-        <v>0.697666772520778</v>
+        <v>0.687699473796195</v>
       </c>
       <c r="T271" s="23" t="n">
         <f aca="false">S271*G271*(1+Hypothèses!$B$22)</f>
-        <v>0.521157079073021</v>
+        <v>0.272328991623293</v>
       </c>
       <c r="U271" s="5" t="s">
         <v>101</v>
@@ -24261,7 +24257,7 @@
         <v>27</v>
       </c>
       <c r="B272" s="21" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C272" s="21" t="s">
         <v>108</v>
@@ -24273,13 +24269,13 @@
         <v>146</v>
       </c>
       <c r="F272" s="21" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="G272" s="22" t="n">
-        <v>0.264</v>
+        <v>2.145</v>
       </c>
       <c r="H272" s="6" t="n">
-        <v>2727</v>
+        <v>2725</v>
       </c>
       <c r="I272" s="23" t="n">
         <f aca="false">IF(A272="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H272,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H272,Hypothèses!$A$6:$A$16,1)))</f>
@@ -24287,7 +24283,7 @@
       </c>
       <c r="J272" s="24" t="n">
         <f aca="false">H272/3600/I272</f>
-        <v>0.137727272727273</v>
+        <v>0.137626262626263</v>
       </c>
       <c r="K272" s="21" t="n">
         <f aca="false">IF(A272="CTA 4",Hypothèses!$B$25,IF(AND(A272="CTA 5",H272&gt;4000),Hypothèses!$B$29,IF(H272&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -24303,7 +24299,7 @@
       </c>
       <c r="N272" s="25" t="n">
         <f aca="false">H272/3600/M272</f>
-        <v>5.05</v>
+        <v>5.0462962962963</v>
       </c>
       <c r="O272" s="21" t="str">
         <f aca="false">IF(N272&lt;=I272,"oui","NON")</f>
@@ -24315,19 +24311,19 @@
       </c>
       <c r="Q272" s="26" t="n">
         <f aca="false">N272*P272/Hypothèses!$B$20</f>
-        <v>141393.033315446</v>
+        <v>141289.334721156</v>
       </c>
       <c r="R272" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P272)+5.74/Q272^0.9))^2</f>
-        <v>0.018875244148939</v>
+        <v>0.0188769675869741</v>
       </c>
       <c r="S272" s="25" t="n">
         <f aca="false">R272/P272*Hypothèses!$B$19*N272^2/2</f>
-        <v>0.687699473796195</v>
+        <v>0.686753816496657</v>
       </c>
       <c r="T272" s="23" t="n">
         <f aca="false">S272*G272*(1+Hypothèses!$B$22)</f>
-        <v>0.272328991623293</v>
+        <v>2.20963040457799</v>
       </c>
       <c r="U272" s="5" t="s">
         <v>101</v>
@@ -24342,7 +24338,7 @@
         <v>27</v>
       </c>
       <c r="B273" s="21" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C273" s="21" t="s">
         <v>108</v>
@@ -24354,13 +24350,13 @@
         <v>146</v>
       </c>
       <c r="F273" s="21" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="G273" s="22" t="n">
-        <v>2.145</v>
+        <v>1.062</v>
       </c>
       <c r="H273" s="6" t="n">
-        <v>2725</v>
+        <v>2720</v>
       </c>
       <c r="I273" s="23" t="n">
         <f aca="false">IF(A273="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H273,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H273,Hypothèses!$A$6:$A$16,1)))</f>
@@ -24368,7 +24364,7 @@
       </c>
       <c r="J273" s="24" t="n">
         <f aca="false">H273/3600/I273</f>
-        <v>0.137626262626263</v>
+        <v>0.137373737373737</v>
       </c>
       <c r="K273" s="21" t="n">
         <f aca="false">IF(A273="CTA 4",Hypothèses!$B$25,IF(AND(A273="CTA 5",H273&gt;4000),Hypothèses!$B$29,IF(H273&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -24384,7 +24380,7 @@
       </c>
       <c r="N273" s="25" t="n">
         <f aca="false">H273/3600/M273</f>
-        <v>5.0462962962963</v>
+        <v>5.03703703703704</v>
       </c>
       <c r="O273" s="21" t="str">
         <f aca="false">IF(N273&lt;=I273,"oui","NON")</f>
@@ -24396,19 +24392,19 @@
       </c>
       <c r="Q273" s="26" t="n">
         <f aca="false">N273*P273/Hypothèses!$B$20</f>
-        <v>141289.334721156</v>
+        <v>141030.088235429</v>
       </c>
       <c r="R273" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P273)+5.74/Q273^0.9))^2</f>
-        <v>0.0188769675869741</v>
+        <v>0.0188812848568492</v>
       </c>
       <c r="S273" s="25" t="n">
         <f aca="false">R273/P273*Hypothèses!$B$19*N273^2/2</f>
-        <v>0.686753816496657</v>
+        <v>0.684392419762669</v>
       </c>
       <c r="T273" s="23" t="n">
         <f aca="false">S273*G273*(1+Hypothèses!$B$22)</f>
-        <v>2.20963040457799</v>
+        <v>1.09023712468193</v>
       </c>
       <c r="U273" s="5" t="s">
         <v>101</v>
@@ -24423,7 +24419,7 @@
         <v>27</v>
       </c>
       <c r="B274" s="21" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C274" s="21" t="s">
         <v>108</v>
@@ -24435,10 +24431,10 @@
         <v>146</v>
       </c>
       <c r="F274" s="21" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="G274" s="22" t="n">
-        <v>1.062</v>
+        <v>1.378</v>
       </c>
       <c r="H274" s="6" t="n">
         <v>2720</v>
@@ -24489,7 +24485,7 @@
       </c>
       <c r="T274" s="23" t="n">
         <f aca="false">S274*G274*(1+Hypothèses!$B$22)</f>
-        <v>1.09023712468193</v>
+        <v>1.41463913164944</v>
       </c>
       <c r="U274" s="5" t="s">
         <v>101</v>
@@ -24504,10 +24500,10 @@
         <v>27</v>
       </c>
       <c r="B275" s="21" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C275" s="21" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D275" s="21" t="s">
         <v>111</v>
@@ -24515,14 +24511,12 @@
       <c r="E275" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="F275" s="21" t="s">
-        <v>362</v>
-      </c>
+      <c r="F275" s="21"/>
       <c r="G275" s="22" t="n">
-        <v>1.378</v>
+        <v>2</v>
       </c>
       <c r="H275" s="6" t="n">
-        <v>2720</v>
+        <v>2030</v>
       </c>
       <c r="I275" s="23" t="n">
         <f aca="false">IF(A275="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H275,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H275,Hypothèses!$A$6:$A$16,1)))</f>
@@ -24530,7 +24524,7 @@
       </c>
       <c r="J275" s="24" t="n">
         <f aca="false">H275/3600/I275</f>
-        <v>0.137373737373737</v>
+        <v>0.102525252525253</v>
       </c>
       <c r="K275" s="21" t="n">
         <f aca="false">IF(A275="CTA 4",Hypothèses!$B$25,IF(AND(A275="CTA 5",H275&gt;4000),Hypothèses!$B$29,IF(H275&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -24538,15 +24532,15 @@
       </c>
       <c r="L275" s="21" t="n">
         <f aca="false">MAX(Hypothèses!$B$26,CEILING(J275/(K275/1000)*1000,Hypothèses!$B$27))</f>
-        <v>500</v>
+        <v>350</v>
       </c>
       <c r="M275" s="24" t="n">
         <f aca="false">L275*K275/1000000</f>
-        <v>0.15</v>
+        <v>0.105</v>
       </c>
       <c r="N275" s="25" t="n">
         <f aca="false">H275/3600/M275</f>
-        <v>5.03703703703704</v>
+        <v>5.37037037037037</v>
       </c>
       <c r="O275" s="21" t="str">
         <f aca="false">IF(N275&lt;=I275,"oui","NON")</f>
@@ -24554,27 +24548,25 @@
       </c>
       <c r="P275" s="24" t="n">
         <f aca="false">1.3*((L275/1000)*(K275/1000))^0.625/((L275/1000)+(K275/1000))^0.25</f>
-        <v>0.419979306877563</v>
+        <v>0.353963373098496</v>
       </c>
       <c r="Q275" s="26" t="n">
         <f aca="false">N275*P275/Hypothèses!$B$20</f>
-        <v>141030.088235429</v>
+        <v>126727.627405634</v>
       </c>
       <c r="R275" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P275)+5.74/Q275^0.9))^2</f>
-        <v>0.0188812848568492</v>
+        <v>0.019473289099905</v>
       </c>
       <c r="S275" s="25" t="n">
         <f aca="false">R275/P275*Hypothèses!$B$19*N275^2/2</f>
-        <v>0.684392419762669</v>
+        <v>0.952008252068462</v>
       </c>
       <c r="T275" s="23" t="n">
         <f aca="false">S275*G275*(1+Hypothèses!$B$22)</f>
-        <v>1.41463913164944</v>
-      </c>
-      <c r="U275" s="5" t="s">
-        <v>101</v>
-      </c>
+        <v>2.85602475620538</v>
+      </c>
+      <c r="U275" s="5"/>
       <c r="V275" s="21" t="str">
         <f aca="false">IF(K275&lt;=Hypothèses!$B$28-100,"oui","NON")</f>
         <v>oui</v>
@@ -24585,7 +24577,7 @@
         <v>27</v>
       </c>
       <c r="B276" s="21" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C276" s="21" t="s">
         <v>104</v>
@@ -24596,9 +24588,11 @@
       <c r="E276" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="F276" s="21"/>
+      <c r="F276" s="21" t="s">
+        <v>422</v>
+      </c>
       <c r="G276" s="22" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="H276" s="6" t="n">
         <v>2030</v>
@@ -24649,7 +24643,7 @@
       </c>
       <c r="T276" s="23" t="n">
         <f aca="false">S276*G276*(1+Hypothèses!$B$22)</f>
-        <v>2.85602475620538</v>
+        <v>1.8564160915335</v>
       </c>
       <c r="U276" s="5"/>
       <c r="V276" s="21" t="str">
@@ -24662,7 +24656,7 @@
         <v>27</v>
       </c>
       <c r="B277" s="21" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="C277" s="21" t="s">
         <v>104</v>
@@ -24674,37 +24668,37 @@
         <v>146</v>
       </c>
       <c r="F277" s="21" t="s">
-        <v>422</v>
+        <v>356</v>
       </c>
       <c r="G277" s="22" t="n">
-        <v>1.3</v>
+        <v>0.475</v>
       </c>
       <c r="H277" s="6" t="n">
-        <v>2030</v>
+        <v>816</v>
       </c>
       <c r="I277" s="23" t="n">
         <f aca="false">IF(A277="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H277,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H277,Hypothèses!$A$6:$A$16,1)))</f>
-        <v>5.5</v>
+        <v>4.5</v>
       </c>
       <c r="J277" s="24" t="n">
         <f aca="false">H277/3600/I277</f>
-        <v>0.102525252525253</v>
+        <v>0.0503703703703704</v>
       </c>
       <c r="K277" s="21" t="n">
         <f aca="false">IF(A277="CTA 4",Hypothèses!$B$25,IF(AND(A277="CTA 5",H277&gt;4000),Hypothèses!$B$29,IF(H277&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="L277" s="21" t="n">
         <f aca="false">MAX(Hypothèses!$B$26,CEILING(J277/(K277/1000)*1000,Hypothèses!$B$27))</f>
-        <v>350</v>
+        <v>250</v>
       </c>
       <c r="M277" s="24" t="n">
         <f aca="false">L277*K277/1000000</f>
-        <v>0.105</v>
+        <v>0.0625</v>
       </c>
       <c r="N277" s="25" t="n">
         <f aca="false">H277/3600/M277</f>
-        <v>5.37037037037037</v>
+        <v>3.62666666666667</v>
       </c>
       <c r="O277" s="21" t="str">
         <f aca="false">IF(N277&lt;=I277,"oui","NON")</f>
@@ -24712,23 +24706,23 @@
       </c>
       <c r="P277" s="24" t="n">
         <f aca="false">1.3*((L277/1000)*(K277/1000))^0.625/((L277/1000)+(K277/1000))^0.25</f>
-        <v>0.353963373098496</v>
+        <v>0.273291334957457</v>
       </c>
       <c r="Q277" s="26" t="n">
         <f aca="false">N277*P277/Hypothèses!$B$20</f>
-        <v>126727.627405634</v>
+        <v>66075.7716519363</v>
       </c>
       <c r="R277" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P277)+5.74/Q277^0.9))^2</f>
-        <v>0.019473289099905</v>
+        <v>0.0218156829546848</v>
       </c>
       <c r="S277" s="25" t="n">
         <f aca="false">R277/P277*Hypothèses!$B$19*N277^2/2</f>
-        <v>0.952008252068462</v>
+        <v>0.629954935759439</v>
       </c>
       <c r="T277" s="23" t="n">
         <f aca="false">S277*G277*(1+Hypothèses!$B$22)</f>
-        <v>1.8564160915335</v>
+        <v>0.4488428917286</v>
       </c>
       <c r="U277" s="5"/>
       <c r="V277" s="21" t="str">
@@ -24741,7 +24735,7 @@
         <v>27</v>
       </c>
       <c r="B278" s="21" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C278" s="21" t="s">
         <v>104</v>
@@ -24753,10 +24747,10 @@
         <v>146</v>
       </c>
       <c r="F278" s="21" t="s">
-        <v>356</v>
+        <v>376</v>
       </c>
       <c r="G278" s="22" t="n">
-        <v>0.475</v>
+        <v>4.281</v>
       </c>
       <c r="H278" s="6" t="n">
         <v>816</v>
@@ -24807,7 +24801,7 @@
       </c>
       <c r="T278" s="23" t="n">
         <f aca="false">S278*G278*(1+Hypothèses!$B$22)</f>
-        <v>0.4488428917286</v>
+        <v>4.04525561997924</v>
       </c>
       <c r="U278" s="5"/>
       <c r="V278" s="21" t="str">
@@ -24820,7 +24814,7 @@
         <v>27</v>
       </c>
       <c r="B279" s="21" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C279" s="21" t="s">
         <v>104</v>
@@ -24832,13 +24826,13 @@
         <v>146</v>
       </c>
       <c r="F279" s="21" t="s">
-        <v>376</v>
+        <v>426</v>
       </c>
       <c r="G279" s="22" t="n">
-        <v>4.281</v>
+        <v>1.294</v>
       </c>
       <c r="H279" s="6" t="n">
-        <v>816</v>
+        <v>814</v>
       </c>
       <c r="I279" s="23" t="n">
         <f aca="false">IF(A279="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H279,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H279,Hypothèses!$A$6:$A$16,1)))</f>
@@ -24846,7 +24840,7 @@
       </c>
       <c r="J279" s="24" t="n">
         <f aca="false">H279/3600/I279</f>
-        <v>0.0503703703703704</v>
+        <v>0.0502469135802469</v>
       </c>
       <c r="K279" s="21" t="n">
         <f aca="false">IF(A279="CTA 4",Hypothèses!$B$25,IF(AND(A279="CTA 5",H279&gt;4000),Hypothèses!$B$29,IF(H279&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
@@ -24862,7 +24856,7 @@
       </c>
       <c r="N279" s="25" t="n">
         <f aca="false">H279/3600/M279</f>
-        <v>3.62666666666667</v>
+        <v>3.61777777777778</v>
       </c>
       <c r="O279" s="21" t="str">
         <f aca="false">IF(N279&lt;=I279,"oui","NON")</f>
@@ -24874,19 +24868,19 @@
       </c>
       <c r="Q279" s="26" t="n">
         <f aca="false">N279*P279/Hypothèses!$B$20</f>
-        <v>66075.7716519363</v>
+        <v>65913.8212312208</v>
       </c>
       <c r="R279" s="27" t="n">
         <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P279)+5.74/Q279^0.9))^2</f>
-        <v>0.0218156829546848</v>
+        <v>0.0218235986157429</v>
       </c>
       <c r="S279" s="25" t="n">
         <f aca="false">R279/P279*Hypothèses!$B$19*N279^2/2</f>
-        <v>0.629954935759439</v>
+        <v>0.627098161152116</v>
       </c>
       <c r="T279" s="23" t="n">
         <f aca="false">S279*G279*(1+Hypothèses!$B$22)</f>
-        <v>4.04525561997924</v>
+        <v>1.21719753079626</v>
       </c>
       <c r="U279" s="5"/>
       <c r="V279" s="21" t="str">
@@ -24894,87 +24888,8 @@
         <v>oui</v>
       </c>
     </row>
-    <row r="280" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A280" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="B280" s="21" t="s">
-        <v>425</v>
-      </c>
-      <c r="C280" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="D280" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="E280" s="21" t="s">
-        <v>146</v>
-      </c>
-      <c r="F280" s="21" t="s">
-        <v>426</v>
-      </c>
-      <c r="G280" s="22" t="n">
-        <v>1.294</v>
-      </c>
-      <c r="H280" s="6" t="n">
-        <v>814</v>
-      </c>
-      <c r="I280" s="23" t="n">
-        <f aca="false">IF(A280="CTA 5",MIN(INDEX(Hypothèses!$C$6:$C$16,MATCH(H280,Hypothèses!$A$6:$A$16,1)),Hypothèses!$B$30),INDEX(Hypothèses!$C$6:$C$16,MATCH(H280,Hypothèses!$A$6:$A$16,1)))</f>
-        <v>4.5</v>
-      </c>
-      <c r="J280" s="24" t="n">
-        <f aca="false">H280/3600/I280</f>
-        <v>0.0502469135802469</v>
-      </c>
-      <c r="K280" s="21" t="n">
-        <f aca="false">IF(A280="CTA 4",Hypothèses!$B$25,IF(AND(A280="CTA 5",H280&gt;4000),Hypothèses!$B$29,IF(H280&lt;=2000,Hypothèses!$B$23,Hypothèses!$B$24)))</f>
-        <v>250</v>
-      </c>
-      <c r="L280" s="21" t="n">
-        <f aca="false">MAX(Hypothèses!$B$26,CEILING(J280/(K280/1000)*1000,Hypothèses!$B$27))</f>
-        <v>250</v>
-      </c>
-      <c r="M280" s="24" t="n">
-        <f aca="false">L280*K280/1000000</f>
-        <v>0.0625</v>
-      </c>
-      <c r="N280" s="25" t="n">
-        <f aca="false">H280/3600/M280</f>
-        <v>3.61777777777778</v>
-      </c>
-      <c r="O280" s="21" t="str">
-        <f aca="false">IF(N280&lt;=I280,"oui","NON")</f>
-        <v>oui</v>
-      </c>
-      <c r="P280" s="24" t="n">
-        <f aca="false">1.3*((L280/1000)*(K280/1000))^0.625/((L280/1000)+(K280/1000))^0.25</f>
-        <v>0.273291334957457</v>
-      </c>
-      <c r="Q280" s="26" t="n">
-        <f aca="false">N280*P280/Hypothèses!$B$20</f>
-        <v>65913.8212312208</v>
-      </c>
-      <c r="R280" s="27" t="n">
-        <f aca="false">0.25/(LOG10(Hypothèses!$B$21/(3.7*P280)+5.74/Q280^0.9))^2</f>
-        <v>0.0218235986157429</v>
-      </c>
-      <c r="S280" s="25" t="n">
-        <f aca="false">R280/P280*Hypothèses!$B$19*N280^2/2</f>
-        <v>0.627098161152116</v>
-      </c>
-      <c r="T280" s="23" t="n">
-        <f aca="false">S280*G280*(1+Hypothèses!$B$22)</f>
-        <v>1.21719753079626</v>
-      </c>
-      <c r="U280" s="5"/>
-      <c r="V280" s="21" t="str">
-        <f aca="false">IF(K280&lt;=Hypothèses!$B$28-100,"oui","NON")</f>
-        <v>oui</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:V280"/>
+  <autoFilter ref="A4:V279"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>